<commit_message>
Fix C14:C73, D14:D73, and G/H/I/J refi trigger row-reference bugs in Debt & Refi sheet
</commit_message>
<xml_diff>
--- a/backend/models/Institutional_Self_Storage_Acquisition_Model_v3_Toggle_Waterfall_Metrics.xlsx
+++ b/backend/models/Institutional_Self_Storage_Acquisition_Model_v3_Toggle_Waterfall_Metrics.xlsx
@@ -14576,11 +14576,11 @@
         <v/>
       </c>
       <c r="C14" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A14&lt;Inputs!$B$28,Inputs!$B$26/12*B14,PMT(Inputs!$B$26/12,Inputs!$B$27*12,-B14)))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A14&lt;Inputs!$B$28,Inputs!$B$27/12*B14,PMT(Inputs!$B$27/12,Inputs!$B$28*12,-B14)))</f>
         <v/>
       </c>
       <c r="D14" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,B14*Inputs!$B$26/12)</f>
+        <f>IF(Inputs!$B$49="Yes",0,B14*Inputs!$B$27/12)</f>
         <v/>
       </c>
       <c r="E14" s="17">
@@ -14592,19 +14592,19 @@
         <v/>
       </c>
       <c r="G14" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A14=Inputs!$B$30,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A14=Inputs!$B$31,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
         <v/>
       </c>
       <c r="H14" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A14=Inputs!$B$30,G14*Inputs!$B$31,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A14=Inputs!$B$31,G14*Inputs!$B$31,0))</f>
         <v/>
       </c>
       <c r="I14" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A14=Inputs!$B$30,MAX(0,H14-F14),0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A14=Inputs!$B$31,MAX(0,H14-F14),0))</f>
         <v/>
       </c>
       <c r="J14" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A14=Inputs!$B$30,H14,F14))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A14=Inputs!$B$31,H14,F14))</f>
         <v/>
       </c>
       <c r="K14" s="1" t="n"/>
@@ -14619,11 +14619,11 @@
         <v/>
       </c>
       <c r="C15" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A15&lt;Inputs!$B$28,Inputs!$B$26/12*B15,PMT(Inputs!$B$26/12,Inputs!$B$27*12,-B15)))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A15&lt;Inputs!$B$28,Inputs!$B$27/12*B15,PMT(Inputs!$B$27/12,Inputs!$B$28*12,-B15)))</f>
         <v/>
       </c>
       <c r="D15" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,B15*Inputs!$B$26/12)</f>
+        <f>IF(Inputs!$B$49="Yes",0,B15*Inputs!$B$27/12)</f>
         <v/>
       </c>
       <c r="E15" s="17">
@@ -14635,19 +14635,19 @@
         <v/>
       </c>
       <c r="G15" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A15=Inputs!$B$30,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A15=Inputs!$B$31,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
         <v/>
       </c>
       <c r="H15" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A15=Inputs!$B$30,G15*Inputs!$B$31,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A15=Inputs!$B$31,G15*Inputs!$B$31,0))</f>
         <v/>
       </c>
       <c r="I15" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A15=Inputs!$B$30,MAX(0,H15-F15),0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A15=Inputs!$B$31,MAX(0,H15-F15),0))</f>
         <v/>
       </c>
       <c r="J15" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A15=Inputs!$B$30,H15,F15))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A15=Inputs!$B$31,H15,F15))</f>
         <v/>
       </c>
       <c r="K15" s="1" t="n"/>
@@ -14662,11 +14662,11 @@
         <v/>
       </c>
       <c r="C16" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A16&lt;Inputs!$B$28,Inputs!$B$26/12*B16,PMT(Inputs!$B$26/12,Inputs!$B$27*12,-B16)))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A16&lt;Inputs!$B$28,Inputs!$B$27/12*B16,PMT(Inputs!$B$27/12,Inputs!$B$28*12,-B16)))</f>
         <v/>
       </c>
       <c r="D16" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,B16*Inputs!$B$26/12)</f>
+        <f>IF(Inputs!$B$49="Yes",0,B16*Inputs!$B$27/12)</f>
         <v/>
       </c>
       <c r="E16" s="17">
@@ -14678,19 +14678,19 @@
         <v/>
       </c>
       <c r="G16" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A16=Inputs!$B$30,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A16=Inputs!$B$31,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
         <v/>
       </c>
       <c r="H16" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A16=Inputs!$B$30,G16*Inputs!$B$31,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A16=Inputs!$B$31,G16*Inputs!$B$31,0))</f>
         <v/>
       </c>
       <c r="I16" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A16=Inputs!$B$30,MAX(0,H16-F16),0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A16=Inputs!$B$31,MAX(0,H16-F16),0))</f>
         <v/>
       </c>
       <c r="J16" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A16=Inputs!$B$30,H16,F16))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A16=Inputs!$B$31,H16,F16))</f>
         <v/>
       </c>
       <c r="K16" s="1" t="n"/>
@@ -14705,11 +14705,11 @@
         <v/>
       </c>
       <c r="C17" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A17&lt;Inputs!$B$28,Inputs!$B$26/12*B17,PMT(Inputs!$B$26/12,Inputs!$B$27*12,-B17)))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A17&lt;Inputs!$B$28,Inputs!$B$27/12*B17,PMT(Inputs!$B$27/12,Inputs!$B$28*12,-B17)))</f>
         <v/>
       </c>
       <c r="D17" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,B17*Inputs!$B$26/12)</f>
+        <f>IF(Inputs!$B$49="Yes",0,B17*Inputs!$B$27/12)</f>
         <v/>
       </c>
       <c r="E17" s="17">
@@ -14721,19 +14721,19 @@
         <v/>
       </c>
       <c r="G17" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A17=Inputs!$B$30,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A17=Inputs!$B$31,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
         <v/>
       </c>
       <c r="H17" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A17=Inputs!$B$30,G17*Inputs!$B$31,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A17=Inputs!$B$31,G17*Inputs!$B$31,0))</f>
         <v/>
       </c>
       <c r="I17" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A17=Inputs!$B$30,MAX(0,H17-F17),0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A17=Inputs!$B$31,MAX(0,H17-F17),0))</f>
         <v/>
       </c>
       <c r="J17" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A17=Inputs!$B$30,H17,F17))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A17=Inputs!$B$31,H17,F17))</f>
         <v/>
       </c>
       <c r="K17" s="1" t="n"/>
@@ -14748,11 +14748,11 @@
         <v/>
       </c>
       <c r="C18" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A18&lt;Inputs!$B$28,Inputs!$B$26/12*B18,PMT(Inputs!$B$26/12,Inputs!$B$27*12,-B18)))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A18&lt;Inputs!$B$28,Inputs!$B$27/12*B18,PMT(Inputs!$B$27/12,Inputs!$B$28*12,-B18)))</f>
         <v/>
       </c>
       <c r="D18" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,B18*Inputs!$B$26/12)</f>
+        <f>IF(Inputs!$B$49="Yes",0,B18*Inputs!$B$27/12)</f>
         <v/>
       </c>
       <c r="E18" s="17">
@@ -14764,19 +14764,19 @@
         <v/>
       </c>
       <c r="G18" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A18=Inputs!$B$30,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A18=Inputs!$B$31,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
         <v/>
       </c>
       <c r="H18" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A18=Inputs!$B$30,G18*Inputs!$B$31,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A18=Inputs!$B$31,G18*Inputs!$B$31,0))</f>
         <v/>
       </c>
       <c r="I18" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A18=Inputs!$B$30,MAX(0,H18-F18),0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A18=Inputs!$B$31,MAX(0,H18-F18),0))</f>
         <v/>
       </c>
       <c r="J18" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A18=Inputs!$B$30,H18,F18))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A18=Inputs!$B$31,H18,F18))</f>
         <v/>
       </c>
       <c r="K18" s="1" t="n"/>
@@ -14791,11 +14791,11 @@
         <v/>
       </c>
       <c r="C19" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A19&lt;Inputs!$B$28,Inputs!$B$26/12*B19,PMT(Inputs!$B$26/12,Inputs!$B$27*12,-B19)))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A19&lt;Inputs!$B$28,Inputs!$B$27/12*B19,PMT(Inputs!$B$27/12,Inputs!$B$28*12,-B19)))</f>
         <v/>
       </c>
       <c r="D19" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,B19*Inputs!$B$26/12)</f>
+        <f>IF(Inputs!$B$49="Yes",0,B19*Inputs!$B$27/12)</f>
         <v/>
       </c>
       <c r="E19" s="17">
@@ -14807,19 +14807,19 @@
         <v/>
       </c>
       <c r="G19" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A19=Inputs!$B$30,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A19=Inputs!$B$31,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
         <v/>
       </c>
       <c r="H19" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A19=Inputs!$B$30,G19*Inputs!$B$31,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A19=Inputs!$B$31,G19*Inputs!$B$31,0))</f>
         <v/>
       </c>
       <c r="I19" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A19=Inputs!$B$30,MAX(0,H19-F19),0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A19=Inputs!$B$31,MAX(0,H19-F19),0))</f>
         <v/>
       </c>
       <c r="J19" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A19=Inputs!$B$30,H19,F19))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A19=Inputs!$B$31,H19,F19))</f>
         <v/>
       </c>
       <c r="K19" s="1" t="n"/>
@@ -14834,11 +14834,11 @@
         <v/>
       </c>
       <c r="C20" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A20&lt;Inputs!$B$28,Inputs!$B$26/12*B20,PMT(Inputs!$B$26/12,Inputs!$B$27*12,-B20)))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A20&lt;Inputs!$B$28,Inputs!$B$27/12*B20,PMT(Inputs!$B$27/12,Inputs!$B$28*12,-B20)))</f>
         <v/>
       </c>
       <c r="D20" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,B20*Inputs!$B$26/12)</f>
+        <f>IF(Inputs!$B$49="Yes",0,B20*Inputs!$B$27/12)</f>
         <v/>
       </c>
       <c r="E20" s="17">
@@ -14850,19 +14850,19 @@
         <v/>
       </c>
       <c r="G20" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A20=Inputs!$B$30,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A20=Inputs!$B$31,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
         <v/>
       </c>
       <c r="H20" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A20=Inputs!$B$30,G20*Inputs!$B$31,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A20=Inputs!$B$31,G20*Inputs!$B$31,0))</f>
         <v/>
       </c>
       <c r="I20" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A20=Inputs!$B$30,MAX(0,H20-F20),0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A20=Inputs!$B$31,MAX(0,H20-F20),0))</f>
         <v/>
       </c>
       <c r="J20" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A20=Inputs!$B$30,H20,F20))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A20=Inputs!$B$31,H20,F20))</f>
         <v/>
       </c>
       <c r="K20" s="1" t="n"/>
@@ -14877,11 +14877,11 @@
         <v/>
       </c>
       <c r="C21" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A21&lt;Inputs!$B$28,Inputs!$B$26/12*B21,PMT(Inputs!$B$26/12,Inputs!$B$27*12,-B21)))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A21&lt;Inputs!$B$28,Inputs!$B$27/12*B21,PMT(Inputs!$B$27/12,Inputs!$B$28*12,-B21)))</f>
         <v/>
       </c>
       <c r="D21" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,B21*Inputs!$B$26/12)</f>
+        <f>IF(Inputs!$B$49="Yes",0,B21*Inputs!$B$27/12)</f>
         <v/>
       </c>
       <c r="E21" s="17">
@@ -14893,19 +14893,19 @@
         <v/>
       </c>
       <c r="G21" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A21=Inputs!$B$30,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A21=Inputs!$B$31,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
         <v/>
       </c>
       <c r="H21" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A21=Inputs!$B$30,G21*Inputs!$B$31,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A21=Inputs!$B$31,G21*Inputs!$B$31,0))</f>
         <v/>
       </c>
       <c r="I21" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A21=Inputs!$B$30,MAX(0,H21-F21),0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A21=Inputs!$B$31,MAX(0,H21-F21),0))</f>
         <v/>
       </c>
       <c r="J21" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A21=Inputs!$B$30,H21,F21))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A21=Inputs!$B$31,H21,F21))</f>
         <v/>
       </c>
       <c r="K21" s="1" t="n"/>
@@ -14920,11 +14920,11 @@
         <v/>
       </c>
       <c r="C22" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A22&lt;Inputs!$B$28,Inputs!$B$26/12*B22,PMT(Inputs!$B$26/12,Inputs!$B$27*12,-B22)))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A22&lt;Inputs!$B$28,Inputs!$B$27/12*B22,PMT(Inputs!$B$27/12,Inputs!$B$28*12,-B22)))</f>
         <v/>
       </c>
       <c r="D22" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,B22*Inputs!$B$26/12)</f>
+        <f>IF(Inputs!$B$49="Yes",0,B22*Inputs!$B$27/12)</f>
         <v/>
       </c>
       <c r="E22" s="17">
@@ -14936,19 +14936,19 @@
         <v/>
       </c>
       <c r="G22" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A22=Inputs!$B$30,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A22=Inputs!$B$31,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
         <v/>
       </c>
       <c r="H22" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A22=Inputs!$B$30,G22*Inputs!$B$31,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A22=Inputs!$B$31,G22*Inputs!$B$31,0))</f>
         <v/>
       </c>
       <c r="I22" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A22=Inputs!$B$30,MAX(0,H22-F22),0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A22=Inputs!$B$31,MAX(0,H22-F22),0))</f>
         <v/>
       </c>
       <c r="J22" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A22=Inputs!$B$30,H22,F22))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A22=Inputs!$B$31,H22,F22))</f>
         <v/>
       </c>
       <c r="K22" s="1" t="n"/>
@@ -14963,11 +14963,11 @@
         <v/>
       </c>
       <c r="C23" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A23&lt;Inputs!$B$28,Inputs!$B$26/12*B23,PMT(Inputs!$B$26/12,Inputs!$B$27*12,-B23)))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A23&lt;Inputs!$B$28,Inputs!$B$27/12*B23,PMT(Inputs!$B$27/12,Inputs!$B$28*12,-B23)))</f>
         <v/>
       </c>
       <c r="D23" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,B23*Inputs!$B$26/12)</f>
+        <f>IF(Inputs!$B$49="Yes",0,B23*Inputs!$B$27/12)</f>
         <v/>
       </c>
       <c r="E23" s="17">
@@ -14979,19 +14979,19 @@
         <v/>
       </c>
       <c r="G23" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A23=Inputs!$B$30,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A23=Inputs!$B$31,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
         <v/>
       </c>
       <c r="H23" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A23=Inputs!$B$30,G23*Inputs!$B$31,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A23=Inputs!$B$31,G23*Inputs!$B$31,0))</f>
         <v/>
       </c>
       <c r="I23" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A23=Inputs!$B$30,MAX(0,H23-F23),0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A23=Inputs!$B$31,MAX(0,H23-F23),0))</f>
         <v/>
       </c>
       <c r="J23" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A23=Inputs!$B$30,H23,F23))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A23=Inputs!$B$31,H23,F23))</f>
         <v/>
       </c>
       <c r="K23" s="1" t="n"/>
@@ -15006,11 +15006,11 @@
         <v/>
       </c>
       <c r="C24" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A24&lt;Inputs!$B$28,Inputs!$B$26/12*B24,PMT(Inputs!$B$26/12,Inputs!$B$27*12,-B24)))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A24&lt;Inputs!$B$28,Inputs!$B$27/12*B24,PMT(Inputs!$B$27/12,Inputs!$B$28*12,-B24)))</f>
         <v/>
       </c>
       <c r="D24" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,B24*Inputs!$B$26/12)</f>
+        <f>IF(Inputs!$B$49="Yes",0,B24*Inputs!$B$27/12)</f>
         <v/>
       </c>
       <c r="E24" s="17">
@@ -15022,19 +15022,19 @@
         <v/>
       </c>
       <c r="G24" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A24=Inputs!$B$30,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A24=Inputs!$B$31,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
         <v/>
       </c>
       <c r="H24" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A24=Inputs!$B$30,G24*Inputs!$B$31,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A24=Inputs!$B$31,G24*Inputs!$B$31,0))</f>
         <v/>
       </c>
       <c r="I24" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A24=Inputs!$B$30,MAX(0,H24-F24),0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A24=Inputs!$B$31,MAX(0,H24-F24),0))</f>
         <v/>
       </c>
       <c r="J24" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A24=Inputs!$B$30,H24,F24))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A24=Inputs!$B$31,H24,F24))</f>
         <v/>
       </c>
       <c r="K24" s="1" t="n"/>
@@ -15049,11 +15049,11 @@
         <v/>
       </c>
       <c r="C25" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A25&lt;Inputs!$B$28,Inputs!$B$26/12*B25,PMT(Inputs!$B$26/12,Inputs!$B$27*12,-B25)))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A25&lt;Inputs!$B$28,Inputs!$B$27/12*B25,PMT(Inputs!$B$27/12,Inputs!$B$28*12,-B25)))</f>
         <v/>
       </c>
       <c r="D25" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,B25*Inputs!$B$26/12)</f>
+        <f>IF(Inputs!$B$49="Yes",0,B25*Inputs!$B$27/12)</f>
         <v/>
       </c>
       <c r="E25" s="17">
@@ -15065,19 +15065,19 @@
         <v/>
       </c>
       <c r="G25" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A25=Inputs!$B$30,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A25=Inputs!$B$31,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
         <v/>
       </c>
       <c r="H25" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A25=Inputs!$B$30,G25*Inputs!$B$31,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A25=Inputs!$B$31,G25*Inputs!$B$31,0))</f>
         <v/>
       </c>
       <c r="I25" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A25=Inputs!$B$30,MAX(0,H25-F25),0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A25=Inputs!$B$31,MAX(0,H25-F25),0))</f>
         <v/>
       </c>
       <c r="J25" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A25=Inputs!$B$30,H25,F25))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A25=Inputs!$B$31,H25,F25))</f>
         <v/>
       </c>
       <c r="K25" s="1" t="n"/>
@@ -15092,11 +15092,11 @@
         <v/>
       </c>
       <c r="C26" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A26&lt;Inputs!$B$28,Inputs!$B$26/12*B26,PMT(Inputs!$B$26/12,Inputs!$B$27*12,-B26)))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A26&lt;Inputs!$B$28,Inputs!$B$27/12*B26,PMT(Inputs!$B$27/12,Inputs!$B$28*12,-B26)))</f>
         <v/>
       </c>
       <c r="D26" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,B26*Inputs!$B$26/12)</f>
+        <f>IF(Inputs!$B$49="Yes",0,B26*Inputs!$B$27/12)</f>
         <v/>
       </c>
       <c r="E26" s="17">
@@ -15108,19 +15108,19 @@
         <v/>
       </c>
       <c r="G26" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A26=Inputs!$B$30,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A26=Inputs!$B$31,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
         <v/>
       </c>
       <c r="H26" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A26=Inputs!$B$30,G26*Inputs!$B$31,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A26=Inputs!$B$31,G26*Inputs!$B$31,0))</f>
         <v/>
       </c>
       <c r="I26" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A26=Inputs!$B$30,MAX(0,H26-F26),0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A26=Inputs!$B$31,MAX(0,H26-F26),0))</f>
         <v/>
       </c>
       <c r="J26" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A26=Inputs!$B$30,H26,F26))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A26=Inputs!$B$31,H26,F26))</f>
         <v/>
       </c>
       <c r="K26" s="1" t="n"/>
@@ -15135,11 +15135,11 @@
         <v/>
       </c>
       <c r="C27" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A27&lt;Inputs!$B$28,Inputs!$B$26/12*B27,PMT(Inputs!$B$26/12,Inputs!$B$27*12,-B27)))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A27&lt;Inputs!$B$28,Inputs!$B$27/12*B27,PMT(Inputs!$B$27/12,Inputs!$B$28*12,-B27)))</f>
         <v/>
       </c>
       <c r="D27" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,B27*Inputs!$B$26/12)</f>
+        <f>IF(Inputs!$B$49="Yes",0,B27*Inputs!$B$27/12)</f>
         <v/>
       </c>
       <c r="E27" s="17">
@@ -15151,19 +15151,19 @@
         <v/>
       </c>
       <c r="G27" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A27=Inputs!$B$30,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A27=Inputs!$B$31,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
         <v/>
       </c>
       <c r="H27" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A27=Inputs!$B$30,G27*Inputs!$B$31,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A27=Inputs!$B$31,G27*Inputs!$B$31,0))</f>
         <v/>
       </c>
       <c r="I27" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A27=Inputs!$B$30,MAX(0,H27-F27),0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A27=Inputs!$B$31,MAX(0,H27-F27),0))</f>
         <v/>
       </c>
       <c r="J27" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A27=Inputs!$B$30,H27,F27))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A27=Inputs!$B$31,H27,F27))</f>
         <v/>
       </c>
       <c r="K27" s="1" t="n"/>
@@ -15178,11 +15178,11 @@
         <v/>
       </c>
       <c r="C28" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A28&lt;Inputs!$B$28,Inputs!$B$26/12*B28,PMT(Inputs!$B$26/12,Inputs!$B$27*12,-B28)))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A28&lt;Inputs!$B$28,Inputs!$B$27/12*B28,PMT(Inputs!$B$27/12,Inputs!$B$28*12,-B28)))</f>
         <v/>
       </c>
       <c r="D28" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,B28*Inputs!$B$26/12)</f>
+        <f>IF(Inputs!$B$49="Yes",0,B28*Inputs!$B$27/12)</f>
         <v/>
       </c>
       <c r="E28" s="17">
@@ -15194,19 +15194,19 @@
         <v/>
       </c>
       <c r="G28" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A28=Inputs!$B$30,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A28=Inputs!$B$31,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
         <v/>
       </c>
       <c r="H28" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A28=Inputs!$B$30,G28*Inputs!$B$31,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A28=Inputs!$B$31,G28*Inputs!$B$31,0))</f>
         <v/>
       </c>
       <c r="I28" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A28=Inputs!$B$30,MAX(0,H28-F28),0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A28=Inputs!$B$31,MAX(0,H28-F28),0))</f>
         <v/>
       </c>
       <c r="J28" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A28=Inputs!$B$30,H28,F28))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A28=Inputs!$B$31,H28,F28))</f>
         <v/>
       </c>
       <c r="K28" s="1" t="n"/>
@@ -15221,11 +15221,11 @@
         <v/>
       </c>
       <c r="C29" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A29&lt;Inputs!$B$28,Inputs!$B$26/12*B29,PMT(Inputs!$B$26/12,Inputs!$B$27*12,-B29)))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A29&lt;Inputs!$B$28,Inputs!$B$27/12*B29,PMT(Inputs!$B$27/12,Inputs!$B$28*12,-B29)))</f>
         <v/>
       </c>
       <c r="D29" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,B29*Inputs!$B$26/12)</f>
+        <f>IF(Inputs!$B$49="Yes",0,B29*Inputs!$B$27/12)</f>
         <v/>
       </c>
       <c r="E29" s="17">
@@ -15237,19 +15237,19 @@
         <v/>
       </c>
       <c r="G29" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A29=Inputs!$B$30,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A29=Inputs!$B$31,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
         <v/>
       </c>
       <c r="H29" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A29=Inputs!$B$30,G29*Inputs!$B$31,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A29=Inputs!$B$31,G29*Inputs!$B$31,0))</f>
         <v/>
       </c>
       <c r="I29" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A29=Inputs!$B$30,MAX(0,H29-F29),0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A29=Inputs!$B$31,MAX(0,H29-F29),0))</f>
         <v/>
       </c>
       <c r="J29" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A29=Inputs!$B$30,H29,F29))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A29=Inputs!$B$31,H29,F29))</f>
         <v/>
       </c>
       <c r="K29" s="1" t="n"/>
@@ -15264,11 +15264,11 @@
         <v/>
       </c>
       <c r="C30" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A30&lt;Inputs!$B$28,Inputs!$B$26/12*B30,PMT(Inputs!$B$26/12,Inputs!$B$27*12,-B30)))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A30&lt;Inputs!$B$28,Inputs!$B$27/12*B30,PMT(Inputs!$B$27/12,Inputs!$B$28*12,-B30)))</f>
         <v/>
       </c>
       <c r="D30" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,B30*Inputs!$B$26/12)</f>
+        <f>IF(Inputs!$B$49="Yes",0,B30*Inputs!$B$27/12)</f>
         <v/>
       </c>
       <c r="E30" s="17">
@@ -15280,19 +15280,19 @@
         <v/>
       </c>
       <c r="G30" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A30=Inputs!$B$30,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A30=Inputs!$B$31,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
         <v/>
       </c>
       <c r="H30" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A30=Inputs!$B$30,G30*Inputs!$B$31,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A30=Inputs!$B$31,G30*Inputs!$B$31,0))</f>
         <v/>
       </c>
       <c r="I30" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A30=Inputs!$B$30,MAX(0,H30-F30),0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A30=Inputs!$B$31,MAX(0,H30-F30),0))</f>
         <v/>
       </c>
       <c r="J30" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A30=Inputs!$B$30,H30,F30))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A30=Inputs!$B$31,H30,F30))</f>
         <v/>
       </c>
       <c r="K30" s="1" t="n"/>
@@ -15307,11 +15307,11 @@
         <v/>
       </c>
       <c r="C31" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A31&lt;Inputs!$B$28,Inputs!$B$26/12*B31,PMT(Inputs!$B$26/12,Inputs!$B$27*12,-B31)))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A31&lt;Inputs!$B$28,Inputs!$B$27/12*B31,PMT(Inputs!$B$27/12,Inputs!$B$28*12,-B31)))</f>
         <v/>
       </c>
       <c r="D31" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,B31*Inputs!$B$26/12)</f>
+        <f>IF(Inputs!$B$49="Yes",0,B31*Inputs!$B$27/12)</f>
         <v/>
       </c>
       <c r="E31" s="17">
@@ -15323,19 +15323,19 @@
         <v/>
       </c>
       <c r="G31" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A31=Inputs!$B$30,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A31=Inputs!$B$31,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
         <v/>
       </c>
       <c r="H31" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A31=Inputs!$B$30,G31*Inputs!$B$31,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A31=Inputs!$B$31,G31*Inputs!$B$31,0))</f>
         <v/>
       </c>
       <c r="I31" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A31=Inputs!$B$30,MAX(0,H31-F31),0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A31=Inputs!$B$31,MAX(0,H31-F31),0))</f>
         <v/>
       </c>
       <c r="J31" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A31=Inputs!$B$30,H31,F31))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A31=Inputs!$B$31,H31,F31))</f>
         <v/>
       </c>
       <c r="K31" s="1" t="n"/>
@@ -15350,11 +15350,11 @@
         <v/>
       </c>
       <c r="C32" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A32&lt;Inputs!$B$28,Inputs!$B$26/12*B32,PMT(Inputs!$B$26/12,Inputs!$B$27*12,-B32)))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A32&lt;Inputs!$B$28,Inputs!$B$27/12*B32,PMT(Inputs!$B$27/12,Inputs!$B$28*12,-B32)))</f>
         <v/>
       </c>
       <c r="D32" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,B32*Inputs!$B$26/12)</f>
+        <f>IF(Inputs!$B$49="Yes",0,B32*Inputs!$B$27/12)</f>
         <v/>
       </c>
       <c r="E32" s="17">
@@ -15366,19 +15366,19 @@
         <v/>
       </c>
       <c r="G32" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A32=Inputs!$B$30,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A32=Inputs!$B$31,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
         <v/>
       </c>
       <c r="H32" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A32=Inputs!$B$30,G32*Inputs!$B$31,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A32=Inputs!$B$31,G32*Inputs!$B$31,0))</f>
         <v/>
       </c>
       <c r="I32" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A32=Inputs!$B$30,MAX(0,H32-F32),0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A32=Inputs!$B$31,MAX(0,H32-F32),0))</f>
         <v/>
       </c>
       <c r="J32" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A32=Inputs!$B$30,H32,F32))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A32=Inputs!$B$31,H32,F32))</f>
         <v/>
       </c>
       <c r="K32" s="1" t="n"/>
@@ -15393,11 +15393,11 @@
         <v/>
       </c>
       <c r="C33" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A33&lt;Inputs!$B$28,Inputs!$B$26/12*B33,PMT(Inputs!$B$26/12,Inputs!$B$27*12,-B33)))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A33&lt;Inputs!$B$28,Inputs!$B$27/12*B33,PMT(Inputs!$B$27/12,Inputs!$B$28*12,-B33)))</f>
         <v/>
       </c>
       <c r="D33" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,B33*Inputs!$B$26/12)</f>
+        <f>IF(Inputs!$B$49="Yes",0,B33*Inputs!$B$27/12)</f>
         <v/>
       </c>
       <c r="E33" s="17">
@@ -15409,19 +15409,19 @@
         <v/>
       </c>
       <c r="G33" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A33=Inputs!$B$30,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A33=Inputs!$B$31,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
         <v/>
       </c>
       <c r="H33" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A33=Inputs!$B$30,G33*Inputs!$B$31,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A33=Inputs!$B$31,G33*Inputs!$B$31,0))</f>
         <v/>
       </c>
       <c r="I33" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A33=Inputs!$B$30,MAX(0,H33-F33),0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A33=Inputs!$B$31,MAX(0,H33-F33),0))</f>
         <v/>
       </c>
       <c r="J33" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A33=Inputs!$B$30,H33,F33))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A33=Inputs!$B$31,H33,F33))</f>
         <v/>
       </c>
       <c r="K33" s="1" t="n"/>
@@ -15436,11 +15436,11 @@
         <v/>
       </c>
       <c r="C34" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A34&lt;Inputs!$B$28,Inputs!$B$26/12*B34,PMT(Inputs!$B$26/12,Inputs!$B$27*12,-B34)))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A34&lt;Inputs!$B$28,Inputs!$B$27/12*B34,PMT(Inputs!$B$27/12,Inputs!$B$28*12,-B34)))</f>
         <v/>
       </c>
       <c r="D34" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,B34*Inputs!$B$26/12)</f>
+        <f>IF(Inputs!$B$49="Yes",0,B34*Inputs!$B$27/12)</f>
         <v/>
       </c>
       <c r="E34" s="17">
@@ -15452,19 +15452,19 @@
         <v/>
       </c>
       <c r="G34" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A34=Inputs!$B$30,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A34=Inputs!$B$31,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
         <v/>
       </c>
       <c r="H34" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A34=Inputs!$B$30,G34*Inputs!$B$31,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A34=Inputs!$B$31,G34*Inputs!$B$31,0))</f>
         <v/>
       </c>
       <c r="I34" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A34=Inputs!$B$30,MAX(0,H34-F34),0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A34=Inputs!$B$31,MAX(0,H34-F34),0))</f>
         <v/>
       </c>
       <c r="J34" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A34=Inputs!$B$30,H34,F34))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A34=Inputs!$B$31,H34,F34))</f>
         <v/>
       </c>
       <c r="K34" s="1" t="n"/>
@@ -15479,11 +15479,11 @@
         <v/>
       </c>
       <c r="C35" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A35&lt;Inputs!$B$28,Inputs!$B$26/12*B35,PMT(Inputs!$B$26/12,Inputs!$B$27*12,-B35)))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A35&lt;Inputs!$B$28,Inputs!$B$27/12*B35,PMT(Inputs!$B$27/12,Inputs!$B$28*12,-B35)))</f>
         <v/>
       </c>
       <c r="D35" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,B35*Inputs!$B$26/12)</f>
+        <f>IF(Inputs!$B$49="Yes",0,B35*Inputs!$B$27/12)</f>
         <v/>
       </c>
       <c r="E35" s="17">
@@ -15495,19 +15495,19 @@
         <v/>
       </c>
       <c r="G35" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A35=Inputs!$B$30,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A35=Inputs!$B$31,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
         <v/>
       </c>
       <c r="H35" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A35=Inputs!$B$30,G35*Inputs!$B$31,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A35=Inputs!$B$31,G35*Inputs!$B$31,0))</f>
         <v/>
       </c>
       <c r="I35" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A35=Inputs!$B$30,MAX(0,H35-F35),0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A35=Inputs!$B$31,MAX(0,H35-F35),0))</f>
         <v/>
       </c>
       <c r="J35" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A35=Inputs!$B$30,H35,F35))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A35=Inputs!$B$31,H35,F35))</f>
         <v/>
       </c>
       <c r="K35" s="1" t="n"/>
@@ -15522,11 +15522,11 @@
         <v/>
       </c>
       <c r="C36" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A36&lt;Inputs!$B$28,Inputs!$B$26/12*B36,PMT(Inputs!$B$26/12,Inputs!$B$27*12,-B36)))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A36&lt;Inputs!$B$28,Inputs!$B$27/12*B36,PMT(Inputs!$B$27/12,Inputs!$B$28*12,-B36)))</f>
         <v/>
       </c>
       <c r="D36" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,B36*Inputs!$B$26/12)</f>
+        <f>IF(Inputs!$B$49="Yes",0,B36*Inputs!$B$27/12)</f>
         <v/>
       </c>
       <c r="E36" s="17">
@@ -15538,19 +15538,19 @@
         <v/>
       </c>
       <c r="G36" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A36=Inputs!$B$30,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A36=Inputs!$B$31,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
         <v/>
       </c>
       <c r="H36" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A36=Inputs!$B$30,G36*Inputs!$B$31,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A36=Inputs!$B$31,G36*Inputs!$B$31,0))</f>
         <v/>
       </c>
       <c r="I36" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A36=Inputs!$B$30,MAX(0,H36-F36),0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A36=Inputs!$B$31,MAX(0,H36-F36),0))</f>
         <v/>
       </c>
       <c r="J36" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A36=Inputs!$B$30,H36,F36))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A36=Inputs!$B$31,H36,F36))</f>
         <v/>
       </c>
       <c r="K36" s="1" t="n"/>
@@ -15565,11 +15565,11 @@
         <v/>
       </c>
       <c r="C37" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A37&lt;Inputs!$B$28,Inputs!$B$26/12*B37,PMT(Inputs!$B$26/12,Inputs!$B$27*12,-B37)))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A37&lt;Inputs!$B$28,Inputs!$B$27/12*B37,PMT(Inputs!$B$27/12,Inputs!$B$28*12,-B37)))</f>
         <v/>
       </c>
       <c r="D37" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,B37*Inputs!$B$26/12)</f>
+        <f>IF(Inputs!$B$49="Yes",0,B37*Inputs!$B$27/12)</f>
         <v/>
       </c>
       <c r="E37" s="17">
@@ -15581,19 +15581,19 @@
         <v/>
       </c>
       <c r="G37" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A37=Inputs!$B$30,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A37=Inputs!$B$31,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
         <v/>
       </c>
       <c r="H37" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A37=Inputs!$B$30,G37*Inputs!$B$31,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A37=Inputs!$B$31,G37*Inputs!$B$31,0))</f>
         <v/>
       </c>
       <c r="I37" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A37=Inputs!$B$30,MAX(0,H37-F37),0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A37=Inputs!$B$31,MAX(0,H37-F37),0))</f>
         <v/>
       </c>
       <c r="J37" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A37=Inputs!$B$30,H37,F37))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A37=Inputs!$B$31,H37,F37))</f>
         <v/>
       </c>
       <c r="K37" s="1" t="n"/>
@@ -15608,11 +15608,11 @@
         <v/>
       </c>
       <c r="C38" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A38&lt;Inputs!$B$28,Inputs!$B$26/12*B38,PMT(Inputs!$B$26/12,Inputs!$B$27*12,-B38)))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A38&lt;Inputs!$B$28,Inputs!$B$27/12*B38,PMT(Inputs!$B$27/12,Inputs!$B$28*12,-B38)))</f>
         <v/>
       </c>
       <c r="D38" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,B38*Inputs!$B$26/12)</f>
+        <f>IF(Inputs!$B$49="Yes",0,B38*Inputs!$B$27/12)</f>
         <v/>
       </c>
       <c r="E38" s="17">
@@ -15624,19 +15624,19 @@
         <v/>
       </c>
       <c r="G38" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A38=Inputs!$B$30,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A38=Inputs!$B$31,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
         <v/>
       </c>
       <c r="H38" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A38=Inputs!$B$30,G38*Inputs!$B$31,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A38=Inputs!$B$31,G38*Inputs!$B$31,0))</f>
         <v/>
       </c>
       <c r="I38" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A38=Inputs!$B$30,MAX(0,H38-F38),0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A38=Inputs!$B$31,MAX(0,H38-F38),0))</f>
         <v/>
       </c>
       <c r="J38" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A38=Inputs!$B$30,H38,F38))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A38=Inputs!$B$31,H38,F38))</f>
         <v/>
       </c>
       <c r="K38" s="1" t="n"/>
@@ -15651,11 +15651,11 @@
         <v/>
       </c>
       <c r="C39" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A39&lt;Inputs!$B$28,Inputs!$B$26/12*B39,PMT(Inputs!$B$26/12,Inputs!$B$27*12,-B39)))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A39&lt;Inputs!$B$28,Inputs!$B$27/12*B39,PMT(Inputs!$B$27/12,Inputs!$B$28*12,-B39)))</f>
         <v/>
       </c>
       <c r="D39" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,B39*Inputs!$B$26/12)</f>
+        <f>IF(Inputs!$B$49="Yes",0,B39*Inputs!$B$27/12)</f>
         <v/>
       </c>
       <c r="E39" s="17">
@@ -15667,19 +15667,19 @@
         <v/>
       </c>
       <c r="G39" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A39=Inputs!$B$30,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A39=Inputs!$B$31,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
         <v/>
       </c>
       <c r="H39" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A39=Inputs!$B$30,G39*Inputs!$B$31,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A39=Inputs!$B$31,G39*Inputs!$B$31,0))</f>
         <v/>
       </c>
       <c r="I39" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A39=Inputs!$B$30,MAX(0,H39-F39),0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A39=Inputs!$B$31,MAX(0,H39-F39),0))</f>
         <v/>
       </c>
       <c r="J39" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A39=Inputs!$B$30,H39,F39))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A39=Inputs!$B$31,H39,F39))</f>
         <v/>
       </c>
       <c r="K39" s="1" t="n"/>
@@ -15694,11 +15694,11 @@
         <v/>
       </c>
       <c r="C40" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A40&lt;Inputs!$B$28,Inputs!$B$26/12*B40,PMT(Inputs!$B$26/12,Inputs!$B$27*12,-B40)))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A40&lt;Inputs!$B$28,Inputs!$B$27/12*B40,PMT(Inputs!$B$27/12,Inputs!$B$28*12,-B40)))</f>
         <v/>
       </c>
       <c r="D40" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,B40*Inputs!$B$26/12)</f>
+        <f>IF(Inputs!$B$49="Yes",0,B40*Inputs!$B$27/12)</f>
         <v/>
       </c>
       <c r="E40" s="17">
@@ -15710,19 +15710,19 @@
         <v/>
       </c>
       <c r="G40" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A40=Inputs!$B$30,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A40=Inputs!$B$31,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
         <v/>
       </c>
       <c r="H40" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A40=Inputs!$B$30,G40*Inputs!$B$31,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A40=Inputs!$B$31,G40*Inputs!$B$31,0))</f>
         <v/>
       </c>
       <c r="I40" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A40=Inputs!$B$30,MAX(0,H40-F40),0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A40=Inputs!$B$31,MAX(0,H40-F40),0))</f>
         <v/>
       </c>
       <c r="J40" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A40=Inputs!$B$30,H40,F40))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A40=Inputs!$B$31,H40,F40))</f>
         <v/>
       </c>
       <c r="K40" s="1" t="n"/>
@@ -15737,11 +15737,11 @@
         <v/>
       </c>
       <c r="C41" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A41&lt;Inputs!$B$28,Inputs!$B$26/12*B41,PMT(Inputs!$B$26/12,Inputs!$B$27*12,-B41)))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A41&lt;Inputs!$B$28,Inputs!$B$27/12*B41,PMT(Inputs!$B$27/12,Inputs!$B$28*12,-B41)))</f>
         <v/>
       </c>
       <c r="D41" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,B41*Inputs!$B$26/12)</f>
+        <f>IF(Inputs!$B$49="Yes",0,B41*Inputs!$B$27/12)</f>
         <v/>
       </c>
       <c r="E41" s="17">
@@ -15753,19 +15753,19 @@
         <v/>
       </c>
       <c r="G41" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A41=Inputs!$B$30,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A41=Inputs!$B$31,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
         <v/>
       </c>
       <c r="H41" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A41=Inputs!$B$30,G41*Inputs!$B$31,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A41=Inputs!$B$31,G41*Inputs!$B$31,0))</f>
         <v/>
       </c>
       <c r="I41" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A41=Inputs!$B$30,MAX(0,H41-F41),0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A41=Inputs!$B$31,MAX(0,H41-F41),0))</f>
         <v/>
       </c>
       <c r="J41" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A41=Inputs!$B$30,H41,F41))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A41=Inputs!$B$31,H41,F41))</f>
         <v/>
       </c>
       <c r="K41" s="1" t="n"/>
@@ -15780,11 +15780,11 @@
         <v/>
       </c>
       <c r="C42" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A42&lt;Inputs!$B$28,Inputs!$B$26/12*B42,PMT(Inputs!$B$26/12,Inputs!$B$27*12,-B42)))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A42&lt;Inputs!$B$28,Inputs!$B$27/12*B42,PMT(Inputs!$B$27/12,Inputs!$B$28*12,-B42)))</f>
         <v/>
       </c>
       <c r="D42" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,B42*Inputs!$B$26/12)</f>
+        <f>IF(Inputs!$B$49="Yes",0,B42*Inputs!$B$27/12)</f>
         <v/>
       </c>
       <c r="E42" s="17">
@@ -15796,19 +15796,19 @@
         <v/>
       </c>
       <c r="G42" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A42=Inputs!$B$30,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A42=Inputs!$B$31,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
         <v/>
       </c>
       <c r="H42" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A42=Inputs!$B$30,G42*Inputs!$B$31,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A42=Inputs!$B$31,G42*Inputs!$B$31,0))</f>
         <v/>
       </c>
       <c r="I42" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A42=Inputs!$B$30,MAX(0,H42-F42),0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A42=Inputs!$B$31,MAX(0,H42-F42),0))</f>
         <v/>
       </c>
       <c r="J42" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A42=Inputs!$B$30,H42,F42))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A42=Inputs!$B$31,H42,F42))</f>
         <v/>
       </c>
       <c r="K42" s="1" t="n"/>
@@ -15823,11 +15823,11 @@
         <v/>
       </c>
       <c r="C43" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A43&lt;Inputs!$B$28,Inputs!$B$26/12*B43,PMT(Inputs!$B$26/12,Inputs!$B$27*12,-B43)))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A43&lt;Inputs!$B$28,Inputs!$B$27/12*B43,PMT(Inputs!$B$27/12,Inputs!$B$28*12,-B43)))</f>
         <v/>
       </c>
       <c r="D43" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,B43*Inputs!$B$26/12)</f>
+        <f>IF(Inputs!$B$49="Yes",0,B43*Inputs!$B$27/12)</f>
         <v/>
       </c>
       <c r="E43" s="17">
@@ -15839,19 +15839,19 @@
         <v/>
       </c>
       <c r="G43" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A43=Inputs!$B$30,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A43=Inputs!$B$31,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
         <v/>
       </c>
       <c r="H43" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A43=Inputs!$B$30,G43*Inputs!$B$31,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A43=Inputs!$B$31,G43*Inputs!$B$31,0))</f>
         <v/>
       </c>
       <c r="I43" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A43=Inputs!$B$30,MAX(0,H43-F43),0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A43=Inputs!$B$31,MAX(0,H43-F43),0))</f>
         <v/>
       </c>
       <c r="J43" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A43=Inputs!$B$30,H43,F43))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A43=Inputs!$B$31,H43,F43))</f>
         <v/>
       </c>
       <c r="K43" s="1" t="n"/>
@@ -15866,11 +15866,11 @@
         <v/>
       </c>
       <c r="C44" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A44&lt;Inputs!$B$28,Inputs!$B$26/12*B44,PMT(Inputs!$B$26/12,Inputs!$B$27*12,-B44)))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A44&lt;Inputs!$B$28,Inputs!$B$27/12*B44,PMT(Inputs!$B$27/12,Inputs!$B$28*12,-B44)))</f>
         <v/>
       </c>
       <c r="D44" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,B44*Inputs!$B$26/12)</f>
+        <f>IF(Inputs!$B$49="Yes",0,B44*Inputs!$B$27/12)</f>
         <v/>
       </c>
       <c r="E44" s="17">
@@ -15882,19 +15882,19 @@
         <v/>
       </c>
       <c r="G44" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A44=Inputs!$B$30,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A44=Inputs!$B$31,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
         <v/>
       </c>
       <c r="H44" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A44=Inputs!$B$30,G44*Inputs!$B$31,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A44=Inputs!$B$31,G44*Inputs!$B$31,0))</f>
         <v/>
       </c>
       <c r="I44" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A44=Inputs!$B$30,MAX(0,H44-F44),0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A44=Inputs!$B$31,MAX(0,H44-F44),0))</f>
         <v/>
       </c>
       <c r="J44" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A44=Inputs!$B$30,H44,F44))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A44=Inputs!$B$31,H44,F44))</f>
         <v/>
       </c>
       <c r="K44" s="1" t="n"/>
@@ -15909,11 +15909,11 @@
         <v/>
       </c>
       <c r="C45" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A45&lt;Inputs!$B$28,Inputs!$B$26/12*B45,PMT(Inputs!$B$26/12,Inputs!$B$27*12,-B45)))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A45&lt;Inputs!$B$28,Inputs!$B$27/12*B45,PMT(Inputs!$B$27/12,Inputs!$B$28*12,-B45)))</f>
         <v/>
       </c>
       <c r="D45" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,B45*Inputs!$B$26/12)</f>
+        <f>IF(Inputs!$B$49="Yes",0,B45*Inputs!$B$27/12)</f>
         <v/>
       </c>
       <c r="E45" s="17">
@@ -15925,19 +15925,19 @@
         <v/>
       </c>
       <c r="G45" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A45=Inputs!$B$30,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A45=Inputs!$B$31,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
         <v/>
       </c>
       <c r="H45" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A45=Inputs!$B$30,G45*Inputs!$B$31,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A45=Inputs!$B$31,G45*Inputs!$B$31,0))</f>
         <v/>
       </c>
       <c r="I45" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A45=Inputs!$B$30,MAX(0,H45-F45),0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A45=Inputs!$B$31,MAX(0,H45-F45),0))</f>
         <v/>
       </c>
       <c r="J45" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A45=Inputs!$B$30,H45,F45))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A45=Inputs!$B$31,H45,F45))</f>
         <v/>
       </c>
       <c r="K45" s="1" t="n"/>
@@ -15952,11 +15952,11 @@
         <v/>
       </c>
       <c r="C46" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A46&lt;Inputs!$B$28,Inputs!$B$26/12*B46,PMT(Inputs!$B$26/12,Inputs!$B$27*12,-B46)))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A46&lt;Inputs!$B$28,Inputs!$B$27/12*B46,PMT(Inputs!$B$27/12,Inputs!$B$28*12,-B46)))</f>
         <v/>
       </c>
       <c r="D46" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,B46*Inputs!$B$26/12)</f>
+        <f>IF(Inputs!$B$49="Yes",0,B46*Inputs!$B$27/12)</f>
         <v/>
       </c>
       <c r="E46" s="17">
@@ -15968,19 +15968,19 @@
         <v/>
       </c>
       <c r="G46" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A46=Inputs!$B$30,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A46=Inputs!$B$31,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
         <v/>
       </c>
       <c r="H46" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A46=Inputs!$B$30,G46*Inputs!$B$31,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A46=Inputs!$B$31,G46*Inputs!$B$31,0))</f>
         <v/>
       </c>
       <c r="I46" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A46=Inputs!$B$30,MAX(0,H46-F46),0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A46=Inputs!$B$31,MAX(0,H46-F46),0))</f>
         <v/>
       </c>
       <c r="J46" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A46=Inputs!$B$30,H46,F46))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A46=Inputs!$B$31,H46,F46))</f>
         <v/>
       </c>
       <c r="K46" s="1" t="n"/>
@@ -15995,11 +15995,11 @@
         <v/>
       </c>
       <c r="C47" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A47&lt;Inputs!$B$28,Inputs!$B$26/12*B47,PMT(Inputs!$B$26/12,Inputs!$B$27*12,-B47)))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A47&lt;Inputs!$B$28,Inputs!$B$27/12*B47,PMT(Inputs!$B$27/12,Inputs!$B$28*12,-B47)))</f>
         <v/>
       </c>
       <c r="D47" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,B47*Inputs!$B$26/12)</f>
+        <f>IF(Inputs!$B$49="Yes",0,B47*Inputs!$B$27/12)</f>
         <v/>
       </c>
       <c r="E47" s="17">
@@ -16011,19 +16011,19 @@
         <v/>
       </c>
       <c r="G47" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A47=Inputs!$B$30,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A47=Inputs!$B$31,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
         <v/>
       </c>
       <c r="H47" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A47=Inputs!$B$30,G47*Inputs!$B$31,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A47=Inputs!$B$31,G47*Inputs!$B$31,0))</f>
         <v/>
       </c>
       <c r="I47" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A47=Inputs!$B$30,MAX(0,H47-F47),0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A47=Inputs!$B$31,MAX(0,H47-F47),0))</f>
         <v/>
       </c>
       <c r="J47" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A47=Inputs!$B$30,H47,F47))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A47=Inputs!$B$31,H47,F47))</f>
         <v/>
       </c>
       <c r="K47" s="1" t="n"/>
@@ -16038,11 +16038,11 @@
         <v/>
       </c>
       <c r="C48" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A48&lt;Inputs!$B$28,Inputs!$B$26/12*B48,PMT(Inputs!$B$26/12,Inputs!$B$27*12,-B48)))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A48&lt;Inputs!$B$28,Inputs!$B$27/12*B48,PMT(Inputs!$B$27/12,Inputs!$B$28*12,-B48)))</f>
         <v/>
       </c>
       <c r="D48" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,B48*Inputs!$B$26/12)</f>
+        <f>IF(Inputs!$B$49="Yes",0,B48*Inputs!$B$27/12)</f>
         <v/>
       </c>
       <c r="E48" s="17">
@@ -16054,19 +16054,19 @@
         <v/>
       </c>
       <c r="G48" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A48=Inputs!$B$30,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A48=Inputs!$B$31,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
         <v/>
       </c>
       <c r="H48" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A48=Inputs!$B$30,G48*Inputs!$B$31,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A48=Inputs!$B$31,G48*Inputs!$B$31,0))</f>
         <v/>
       </c>
       <c r="I48" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A48=Inputs!$B$30,MAX(0,H48-F48),0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A48=Inputs!$B$31,MAX(0,H48-F48),0))</f>
         <v/>
       </c>
       <c r="J48" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A48=Inputs!$B$30,H48,F48))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A48=Inputs!$B$31,H48,F48))</f>
         <v/>
       </c>
       <c r="K48" s="1" t="n"/>
@@ -16081,11 +16081,11 @@
         <v/>
       </c>
       <c r="C49" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A49&lt;Inputs!$B$28,Inputs!$B$26/12*B49,PMT(Inputs!$B$26/12,Inputs!$B$27*12,-B49)))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A49&lt;Inputs!$B$28,Inputs!$B$27/12*B49,PMT(Inputs!$B$27/12,Inputs!$B$28*12,-B49)))</f>
         <v/>
       </c>
       <c r="D49" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,B49*Inputs!$B$26/12)</f>
+        <f>IF(Inputs!$B$49="Yes",0,B49*Inputs!$B$27/12)</f>
         <v/>
       </c>
       <c r="E49" s="17">
@@ -16097,19 +16097,19 @@
         <v/>
       </c>
       <c r="G49" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A49=Inputs!$B$30,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A49=Inputs!$B$31,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
         <v/>
       </c>
       <c r="H49" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A49=Inputs!$B$30,G49*Inputs!$B$31,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A49=Inputs!$B$31,G49*Inputs!$B$31,0))</f>
         <v/>
       </c>
       <c r="I49" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A49=Inputs!$B$30,MAX(0,H49-F49),0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A49=Inputs!$B$31,MAX(0,H49-F49),0))</f>
         <v/>
       </c>
       <c r="J49" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A49=Inputs!$B$30,H49,F49))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A49=Inputs!$B$31,H49,F49))</f>
         <v/>
       </c>
       <c r="K49" s="1" t="n"/>
@@ -16124,11 +16124,11 @@
         <v/>
       </c>
       <c r="C50" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A50&lt;Inputs!$B$28,Inputs!$B$26/12*B50,PMT(Inputs!$B$26/12,Inputs!$B$27*12,-B50)))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A50&lt;Inputs!$B$28,Inputs!$B$27/12*B50,PMT(Inputs!$B$27/12,Inputs!$B$28*12,-B50)))</f>
         <v/>
       </c>
       <c r="D50" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,B50*Inputs!$B$26/12)</f>
+        <f>IF(Inputs!$B$49="Yes",0,B50*Inputs!$B$27/12)</f>
         <v/>
       </c>
       <c r="E50" s="17">
@@ -16140,19 +16140,19 @@
         <v/>
       </c>
       <c r="G50" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A50=Inputs!$B$30,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A50=Inputs!$B$31,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
         <v/>
       </c>
       <c r="H50" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A50=Inputs!$B$30,G50*Inputs!$B$31,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A50=Inputs!$B$31,G50*Inputs!$B$31,0))</f>
         <v/>
       </c>
       <c r="I50" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A50=Inputs!$B$30,MAX(0,H50-F50),0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A50=Inputs!$B$31,MAX(0,H50-F50),0))</f>
         <v/>
       </c>
       <c r="J50" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A50=Inputs!$B$30,H50,F50))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A50=Inputs!$B$31,H50,F50))</f>
         <v/>
       </c>
       <c r="K50" s="1" t="n"/>
@@ -16167,11 +16167,11 @@
         <v/>
       </c>
       <c r="C51" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A51&lt;Inputs!$B$28,Inputs!$B$26/12*B51,PMT(Inputs!$B$26/12,Inputs!$B$27*12,-B51)))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A51&lt;Inputs!$B$28,Inputs!$B$27/12*B51,PMT(Inputs!$B$27/12,Inputs!$B$28*12,-B51)))</f>
         <v/>
       </c>
       <c r="D51" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,B51*Inputs!$B$26/12)</f>
+        <f>IF(Inputs!$B$49="Yes",0,B51*Inputs!$B$27/12)</f>
         <v/>
       </c>
       <c r="E51" s="17">
@@ -16183,19 +16183,19 @@
         <v/>
       </c>
       <c r="G51" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A51=Inputs!$B$30,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A51=Inputs!$B$31,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
         <v/>
       </c>
       <c r="H51" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A51=Inputs!$B$30,G51*Inputs!$B$31,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A51=Inputs!$B$31,G51*Inputs!$B$31,0))</f>
         <v/>
       </c>
       <c r="I51" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A51=Inputs!$B$30,MAX(0,H51-F51),0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A51=Inputs!$B$31,MAX(0,H51-F51),0))</f>
         <v/>
       </c>
       <c r="J51" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A51=Inputs!$B$30,H51,F51))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A51=Inputs!$B$31,H51,F51))</f>
         <v/>
       </c>
       <c r="K51" s="1" t="n"/>
@@ -16210,11 +16210,11 @@
         <v/>
       </c>
       <c r="C52" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A52&lt;Inputs!$B$28,Inputs!$B$26/12*B52,PMT(Inputs!$B$26/12,Inputs!$B$27*12,-B52)))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A52&lt;Inputs!$B$28,Inputs!$B$27/12*B52,PMT(Inputs!$B$27/12,Inputs!$B$28*12,-B52)))</f>
         <v/>
       </c>
       <c r="D52" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,B52*Inputs!$B$26/12)</f>
+        <f>IF(Inputs!$B$49="Yes",0,B52*Inputs!$B$27/12)</f>
         <v/>
       </c>
       <c r="E52" s="17">
@@ -16226,19 +16226,19 @@
         <v/>
       </c>
       <c r="G52" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A52=Inputs!$B$30,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A52=Inputs!$B$31,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
         <v/>
       </c>
       <c r="H52" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A52=Inputs!$B$30,G52*Inputs!$B$31,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A52=Inputs!$B$31,G52*Inputs!$B$31,0))</f>
         <v/>
       </c>
       <c r="I52" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A52=Inputs!$B$30,MAX(0,H52-F52),0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A52=Inputs!$B$31,MAX(0,H52-F52),0))</f>
         <v/>
       </c>
       <c r="J52" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A52=Inputs!$B$30,H52,F52))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A52=Inputs!$B$31,H52,F52))</f>
         <v/>
       </c>
       <c r="K52" s="1" t="n"/>
@@ -16253,11 +16253,11 @@
         <v/>
       </c>
       <c r="C53" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A53&lt;Inputs!$B$28,Inputs!$B$26/12*B53,PMT(Inputs!$B$26/12,Inputs!$B$27*12,-B53)))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A53&lt;Inputs!$B$28,Inputs!$B$27/12*B53,PMT(Inputs!$B$27/12,Inputs!$B$28*12,-B53)))</f>
         <v/>
       </c>
       <c r="D53" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,B53*Inputs!$B$26/12)</f>
+        <f>IF(Inputs!$B$49="Yes",0,B53*Inputs!$B$27/12)</f>
         <v/>
       </c>
       <c r="E53" s="17">
@@ -16269,19 +16269,19 @@
         <v/>
       </c>
       <c r="G53" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A53=Inputs!$B$30,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A53=Inputs!$B$31,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
         <v/>
       </c>
       <c r="H53" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A53=Inputs!$B$30,G53*Inputs!$B$31,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A53=Inputs!$B$31,G53*Inputs!$B$31,0))</f>
         <v/>
       </c>
       <c r="I53" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A53=Inputs!$B$30,MAX(0,H53-F53),0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A53=Inputs!$B$31,MAX(0,H53-F53),0))</f>
         <v/>
       </c>
       <c r="J53" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A53=Inputs!$B$30,H53,F53))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A53=Inputs!$B$31,H53,F53))</f>
         <v/>
       </c>
       <c r="K53" s="1" t="n"/>
@@ -16296,11 +16296,11 @@
         <v/>
       </c>
       <c r="C54" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A54&lt;Inputs!$B$28,Inputs!$B$26/12*B54,PMT(Inputs!$B$26/12,Inputs!$B$27*12,-B54)))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A54&lt;Inputs!$B$28,Inputs!$B$27/12*B54,PMT(Inputs!$B$27/12,Inputs!$B$28*12,-B54)))</f>
         <v/>
       </c>
       <c r="D54" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,B54*Inputs!$B$26/12)</f>
+        <f>IF(Inputs!$B$49="Yes",0,B54*Inputs!$B$27/12)</f>
         <v/>
       </c>
       <c r="E54" s="17">
@@ -16312,19 +16312,19 @@
         <v/>
       </c>
       <c r="G54" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A54=Inputs!$B$30,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A54=Inputs!$B$31,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
         <v/>
       </c>
       <c r="H54" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A54=Inputs!$B$30,G54*Inputs!$B$31,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A54=Inputs!$B$31,G54*Inputs!$B$31,0))</f>
         <v/>
       </c>
       <c r="I54" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A54=Inputs!$B$30,MAX(0,H54-F54),0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A54=Inputs!$B$31,MAX(0,H54-F54),0))</f>
         <v/>
       </c>
       <c r="J54" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A54=Inputs!$B$30,H54,F54))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A54=Inputs!$B$31,H54,F54))</f>
         <v/>
       </c>
       <c r="K54" s="1" t="n"/>
@@ -16339,11 +16339,11 @@
         <v/>
       </c>
       <c r="C55" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A55&lt;Inputs!$B$28,Inputs!$B$26/12*B55,PMT(Inputs!$B$26/12,Inputs!$B$27*12,-B55)))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A55&lt;Inputs!$B$28,Inputs!$B$27/12*B55,PMT(Inputs!$B$27/12,Inputs!$B$28*12,-B55)))</f>
         <v/>
       </c>
       <c r="D55" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,B55*Inputs!$B$26/12)</f>
+        <f>IF(Inputs!$B$49="Yes",0,B55*Inputs!$B$27/12)</f>
         <v/>
       </c>
       <c r="E55" s="17">
@@ -16355,19 +16355,19 @@
         <v/>
       </c>
       <c r="G55" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A55=Inputs!$B$30,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A55=Inputs!$B$31,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
         <v/>
       </c>
       <c r="H55" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A55=Inputs!$B$30,G55*Inputs!$B$31,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A55=Inputs!$B$31,G55*Inputs!$B$31,0))</f>
         <v/>
       </c>
       <c r="I55" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A55=Inputs!$B$30,MAX(0,H55-F55),0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A55=Inputs!$B$31,MAX(0,H55-F55),0))</f>
         <v/>
       </c>
       <c r="J55" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A55=Inputs!$B$30,H55,F55))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A55=Inputs!$B$31,H55,F55))</f>
         <v/>
       </c>
       <c r="K55" s="1" t="n"/>
@@ -16382,11 +16382,11 @@
         <v/>
       </c>
       <c r="C56" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A56&lt;Inputs!$B$28,Inputs!$B$26/12*B56,PMT(Inputs!$B$26/12,Inputs!$B$27*12,-B56)))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A56&lt;Inputs!$B$28,Inputs!$B$27/12*B56,PMT(Inputs!$B$27/12,Inputs!$B$28*12,-B56)))</f>
         <v/>
       </c>
       <c r="D56" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,B56*Inputs!$B$26/12)</f>
+        <f>IF(Inputs!$B$49="Yes",0,B56*Inputs!$B$27/12)</f>
         <v/>
       </c>
       <c r="E56" s="17">
@@ -16398,19 +16398,19 @@
         <v/>
       </c>
       <c r="G56" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A56=Inputs!$B$30,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A56=Inputs!$B$31,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
         <v/>
       </c>
       <c r="H56" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A56=Inputs!$B$30,G56*Inputs!$B$31,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A56=Inputs!$B$31,G56*Inputs!$B$31,0))</f>
         <v/>
       </c>
       <c r="I56" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A56=Inputs!$B$30,MAX(0,H56-F56),0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A56=Inputs!$B$31,MAX(0,H56-F56),0))</f>
         <v/>
       </c>
       <c r="J56" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A56=Inputs!$B$30,H56,F56))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A56=Inputs!$B$31,H56,F56))</f>
         <v/>
       </c>
       <c r="K56" s="1" t="n"/>
@@ -16425,11 +16425,11 @@
         <v/>
       </c>
       <c r="C57" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A57&lt;Inputs!$B$28,Inputs!$B$26/12*B57,PMT(Inputs!$B$26/12,Inputs!$B$27*12,-B57)))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A57&lt;Inputs!$B$28,Inputs!$B$27/12*B57,PMT(Inputs!$B$27/12,Inputs!$B$28*12,-B57)))</f>
         <v/>
       </c>
       <c r="D57" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,B57*Inputs!$B$26/12)</f>
+        <f>IF(Inputs!$B$49="Yes",0,B57*Inputs!$B$27/12)</f>
         <v/>
       </c>
       <c r="E57" s="17">
@@ -16441,19 +16441,19 @@
         <v/>
       </c>
       <c r="G57" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A57=Inputs!$B$30,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A57=Inputs!$B$31,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
         <v/>
       </c>
       <c r="H57" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A57=Inputs!$B$30,G57*Inputs!$B$31,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A57=Inputs!$B$31,G57*Inputs!$B$31,0))</f>
         <v/>
       </c>
       <c r="I57" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A57=Inputs!$B$30,MAX(0,H57-F57),0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A57=Inputs!$B$31,MAX(0,H57-F57),0))</f>
         <v/>
       </c>
       <c r="J57" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A57=Inputs!$B$30,H57,F57))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A57=Inputs!$B$31,H57,F57))</f>
         <v/>
       </c>
       <c r="K57" s="1" t="n"/>
@@ -16468,11 +16468,11 @@
         <v/>
       </c>
       <c r="C58" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A58&lt;Inputs!$B$28,Inputs!$B$26/12*B58,PMT(Inputs!$B$26/12,Inputs!$B$27*12,-B58)))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A58&lt;Inputs!$B$28,Inputs!$B$27/12*B58,PMT(Inputs!$B$27/12,Inputs!$B$28*12,-B58)))</f>
         <v/>
       </c>
       <c r="D58" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,B58*Inputs!$B$26/12)</f>
+        <f>IF(Inputs!$B$49="Yes",0,B58*Inputs!$B$27/12)</f>
         <v/>
       </c>
       <c r="E58" s="17">
@@ -16484,19 +16484,19 @@
         <v/>
       </c>
       <c r="G58" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A58=Inputs!$B$30,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A58=Inputs!$B$31,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
         <v/>
       </c>
       <c r="H58" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A58=Inputs!$B$30,G58*Inputs!$B$31,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A58=Inputs!$B$31,G58*Inputs!$B$31,0))</f>
         <v/>
       </c>
       <c r="I58" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A58=Inputs!$B$30,MAX(0,H58-F58),0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A58=Inputs!$B$31,MAX(0,H58-F58),0))</f>
         <v/>
       </c>
       <c r="J58" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A58=Inputs!$B$30,H58,F58))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A58=Inputs!$B$31,H58,F58))</f>
         <v/>
       </c>
       <c r="K58" s="1" t="n"/>
@@ -16511,11 +16511,11 @@
         <v/>
       </c>
       <c r="C59" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A59&lt;Inputs!$B$28,Inputs!$B$26/12*B59,PMT(Inputs!$B$26/12,Inputs!$B$27*12,-B59)))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A59&lt;Inputs!$B$28,Inputs!$B$27/12*B59,PMT(Inputs!$B$27/12,Inputs!$B$28*12,-B59)))</f>
         <v/>
       </c>
       <c r="D59" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,B59*Inputs!$B$26/12)</f>
+        <f>IF(Inputs!$B$49="Yes",0,B59*Inputs!$B$27/12)</f>
         <v/>
       </c>
       <c r="E59" s="17">
@@ -16527,19 +16527,19 @@
         <v/>
       </c>
       <c r="G59" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A59=Inputs!$B$30,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A59=Inputs!$B$31,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
         <v/>
       </c>
       <c r="H59" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A59=Inputs!$B$30,G59*Inputs!$B$31,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A59=Inputs!$B$31,G59*Inputs!$B$31,0))</f>
         <v/>
       </c>
       <c r="I59" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A59=Inputs!$B$30,MAX(0,H59-F59),0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A59=Inputs!$B$31,MAX(0,H59-F59),0))</f>
         <v/>
       </c>
       <c r="J59" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A59=Inputs!$B$30,H59,F59))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A59=Inputs!$B$31,H59,F59))</f>
         <v/>
       </c>
       <c r="K59" s="1" t="n"/>
@@ -16554,11 +16554,11 @@
         <v/>
       </c>
       <c r="C60" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A60&lt;Inputs!$B$28,Inputs!$B$26/12*B60,PMT(Inputs!$B$26/12,Inputs!$B$27*12,-B60)))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A60&lt;Inputs!$B$28,Inputs!$B$27/12*B60,PMT(Inputs!$B$27/12,Inputs!$B$28*12,-B60)))</f>
         <v/>
       </c>
       <c r="D60" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,B60*Inputs!$B$26/12)</f>
+        <f>IF(Inputs!$B$49="Yes",0,B60*Inputs!$B$27/12)</f>
         <v/>
       </c>
       <c r="E60" s="17">
@@ -16570,19 +16570,19 @@
         <v/>
       </c>
       <c r="G60" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A60=Inputs!$B$30,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A60=Inputs!$B$31,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
         <v/>
       </c>
       <c r="H60" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A60=Inputs!$B$30,G60*Inputs!$B$31,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A60=Inputs!$B$31,G60*Inputs!$B$31,0))</f>
         <v/>
       </c>
       <c r="I60" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A60=Inputs!$B$30,MAX(0,H60-F60),0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A60=Inputs!$B$31,MAX(0,H60-F60),0))</f>
         <v/>
       </c>
       <c r="J60" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A60=Inputs!$B$30,H60,F60))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A60=Inputs!$B$31,H60,F60))</f>
         <v/>
       </c>
       <c r="K60" s="1" t="n"/>
@@ -16597,11 +16597,11 @@
         <v/>
       </c>
       <c r="C61" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A61&lt;Inputs!$B$28,Inputs!$B$26/12*B61,PMT(Inputs!$B$26/12,Inputs!$B$27*12,-B61)))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A61&lt;Inputs!$B$28,Inputs!$B$27/12*B61,PMT(Inputs!$B$27/12,Inputs!$B$28*12,-B61)))</f>
         <v/>
       </c>
       <c r="D61" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,B61*Inputs!$B$26/12)</f>
+        <f>IF(Inputs!$B$49="Yes",0,B61*Inputs!$B$27/12)</f>
         <v/>
       </c>
       <c r="E61" s="17">
@@ -16613,19 +16613,19 @@
         <v/>
       </c>
       <c r="G61" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A61=Inputs!$B$30,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A61=Inputs!$B$31,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
         <v/>
       </c>
       <c r="H61" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A61=Inputs!$B$30,G61*Inputs!$B$31,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A61=Inputs!$B$31,G61*Inputs!$B$31,0))</f>
         <v/>
       </c>
       <c r="I61" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A61=Inputs!$B$30,MAX(0,H61-F61),0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A61=Inputs!$B$31,MAX(0,H61-F61),0))</f>
         <v/>
       </c>
       <c r="J61" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A61=Inputs!$B$30,H61,F61))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A61=Inputs!$B$31,H61,F61))</f>
         <v/>
       </c>
       <c r="K61" s="1" t="n"/>
@@ -16640,11 +16640,11 @@
         <v/>
       </c>
       <c r="C62" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A62&lt;Inputs!$B$28,Inputs!$B$26/12*B62,PMT(Inputs!$B$26/12,Inputs!$B$27*12,-B62)))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A62&lt;Inputs!$B$28,Inputs!$B$27/12*B62,PMT(Inputs!$B$27/12,Inputs!$B$28*12,-B62)))</f>
         <v/>
       </c>
       <c r="D62" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,B62*Inputs!$B$26/12)</f>
+        <f>IF(Inputs!$B$49="Yes",0,B62*Inputs!$B$27/12)</f>
         <v/>
       </c>
       <c r="E62" s="17">
@@ -16656,19 +16656,19 @@
         <v/>
       </c>
       <c r="G62" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A62=Inputs!$B$30,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A62=Inputs!$B$31,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
         <v/>
       </c>
       <c r="H62" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A62=Inputs!$B$30,G62*Inputs!$B$31,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A62=Inputs!$B$31,G62*Inputs!$B$31,0))</f>
         <v/>
       </c>
       <c r="I62" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A62=Inputs!$B$30,MAX(0,H62-F62),0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A62=Inputs!$B$31,MAX(0,H62-F62),0))</f>
         <v/>
       </c>
       <c r="J62" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A62=Inputs!$B$30,H62,F62))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A62=Inputs!$B$31,H62,F62))</f>
         <v/>
       </c>
       <c r="K62" s="1" t="n"/>
@@ -16683,11 +16683,11 @@
         <v/>
       </c>
       <c r="C63" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A63&lt;Inputs!$B$28,Inputs!$B$26/12*B63,PMT(Inputs!$B$26/12,Inputs!$B$27*12,-B63)))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A63&lt;Inputs!$B$28,Inputs!$B$27/12*B63,PMT(Inputs!$B$27/12,Inputs!$B$28*12,-B63)))</f>
         <v/>
       </c>
       <c r="D63" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,B63*Inputs!$B$26/12)</f>
+        <f>IF(Inputs!$B$49="Yes",0,B63*Inputs!$B$27/12)</f>
         <v/>
       </c>
       <c r="E63" s="17">
@@ -16699,19 +16699,19 @@
         <v/>
       </c>
       <c r="G63" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A63=Inputs!$B$30,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A63=Inputs!$B$31,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
         <v/>
       </c>
       <c r="H63" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A63=Inputs!$B$30,G63*Inputs!$B$31,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A63=Inputs!$B$31,G63*Inputs!$B$31,0))</f>
         <v/>
       </c>
       <c r="I63" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A63=Inputs!$B$30,MAX(0,H63-F63),0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A63=Inputs!$B$31,MAX(0,H63-F63),0))</f>
         <v/>
       </c>
       <c r="J63" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A63=Inputs!$B$30,H63,F63))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A63=Inputs!$B$31,H63,F63))</f>
         <v/>
       </c>
       <c r="K63" s="1" t="n"/>
@@ -16726,11 +16726,11 @@
         <v/>
       </c>
       <c r="C64" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A64&lt;Inputs!$B$28,Inputs!$B$26/12*B64,PMT(Inputs!$B$26/12,Inputs!$B$27*12,-B64)))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A64&lt;Inputs!$B$28,Inputs!$B$27/12*B64,PMT(Inputs!$B$27/12,Inputs!$B$28*12,-B64)))</f>
         <v/>
       </c>
       <c r="D64" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,B64*Inputs!$B$26/12)</f>
+        <f>IF(Inputs!$B$49="Yes",0,B64*Inputs!$B$27/12)</f>
         <v/>
       </c>
       <c r="E64" s="17">
@@ -16742,19 +16742,19 @@
         <v/>
       </c>
       <c r="G64" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A64=Inputs!$B$30,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A64=Inputs!$B$31,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
         <v/>
       </c>
       <c r="H64" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A64=Inputs!$B$30,G64*Inputs!$B$31,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A64=Inputs!$B$31,G64*Inputs!$B$31,0))</f>
         <v/>
       </c>
       <c r="I64" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A64=Inputs!$B$30,MAX(0,H64-F64),0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A64=Inputs!$B$31,MAX(0,H64-F64),0))</f>
         <v/>
       </c>
       <c r="J64" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A64=Inputs!$B$30,H64,F64))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A64=Inputs!$B$31,H64,F64))</f>
         <v/>
       </c>
       <c r="K64" s="1" t="n"/>
@@ -16769,11 +16769,11 @@
         <v/>
       </c>
       <c r="C65" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A65&lt;Inputs!$B$28,Inputs!$B$26/12*B65,PMT(Inputs!$B$26/12,Inputs!$B$27*12,-B65)))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A65&lt;Inputs!$B$28,Inputs!$B$27/12*B65,PMT(Inputs!$B$27/12,Inputs!$B$28*12,-B65)))</f>
         <v/>
       </c>
       <c r="D65" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,B65*Inputs!$B$26/12)</f>
+        <f>IF(Inputs!$B$49="Yes",0,B65*Inputs!$B$27/12)</f>
         <v/>
       </c>
       <c r="E65" s="17">
@@ -16785,19 +16785,19 @@
         <v/>
       </c>
       <c r="G65" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A65=Inputs!$B$30,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A65=Inputs!$B$31,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
         <v/>
       </c>
       <c r="H65" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A65=Inputs!$B$30,G65*Inputs!$B$31,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A65=Inputs!$B$31,G65*Inputs!$B$31,0))</f>
         <v/>
       </c>
       <c r="I65" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A65=Inputs!$B$30,MAX(0,H65-F65),0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A65=Inputs!$B$31,MAX(0,H65-F65),0))</f>
         <v/>
       </c>
       <c r="J65" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A65=Inputs!$B$30,H65,F65))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A65=Inputs!$B$31,H65,F65))</f>
         <v/>
       </c>
       <c r="K65" s="1" t="n"/>
@@ -16812,11 +16812,11 @@
         <v/>
       </c>
       <c r="C66" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A66&lt;Inputs!$B$28,Inputs!$B$26/12*B66,PMT(Inputs!$B$26/12,Inputs!$B$27*12,-B66)))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A66&lt;Inputs!$B$28,Inputs!$B$27/12*B66,PMT(Inputs!$B$27/12,Inputs!$B$28*12,-B66)))</f>
         <v/>
       </c>
       <c r="D66" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,B66*Inputs!$B$26/12)</f>
+        <f>IF(Inputs!$B$49="Yes",0,B66*Inputs!$B$27/12)</f>
         <v/>
       </c>
       <c r="E66" s="17">
@@ -16828,19 +16828,19 @@
         <v/>
       </c>
       <c r="G66" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A66=Inputs!$B$30,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A66=Inputs!$B$31,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
         <v/>
       </c>
       <c r="H66" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A66=Inputs!$B$30,G66*Inputs!$B$31,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A66=Inputs!$B$31,G66*Inputs!$B$31,0))</f>
         <v/>
       </c>
       <c r="I66" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A66=Inputs!$B$30,MAX(0,H66-F66),0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A66=Inputs!$B$31,MAX(0,H66-F66),0))</f>
         <v/>
       </c>
       <c r="J66" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A66=Inputs!$B$30,H66,F66))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A66=Inputs!$B$31,H66,F66))</f>
         <v/>
       </c>
       <c r="K66" s="1" t="n"/>
@@ -16855,11 +16855,11 @@
         <v/>
       </c>
       <c r="C67" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A67&lt;Inputs!$B$28,Inputs!$B$26/12*B67,PMT(Inputs!$B$26/12,Inputs!$B$27*12,-B67)))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A67&lt;Inputs!$B$28,Inputs!$B$27/12*B67,PMT(Inputs!$B$27/12,Inputs!$B$28*12,-B67)))</f>
         <v/>
       </c>
       <c r="D67" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,B67*Inputs!$B$26/12)</f>
+        <f>IF(Inputs!$B$49="Yes",0,B67*Inputs!$B$27/12)</f>
         <v/>
       </c>
       <c r="E67" s="17">
@@ -16871,19 +16871,19 @@
         <v/>
       </c>
       <c r="G67" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A67=Inputs!$B$30,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A67=Inputs!$B$31,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
         <v/>
       </c>
       <c r="H67" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A67=Inputs!$B$30,G67*Inputs!$B$31,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A67=Inputs!$B$31,G67*Inputs!$B$31,0))</f>
         <v/>
       </c>
       <c r="I67" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A67=Inputs!$B$30,MAX(0,H67-F67),0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A67=Inputs!$B$31,MAX(0,H67-F67),0))</f>
         <v/>
       </c>
       <c r="J67" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A67=Inputs!$B$30,H67,F67))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A67=Inputs!$B$31,H67,F67))</f>
         <v/>
       </c>
       <c r="K67" s="1" t="n"/>
@@ -16898,11 +16898,11 @@
         <v/>
       </c>
       <c r="C68" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A68&lt;Inputs!$B$28,Inputs!$B$26/12*B68,PMT(Inputs!$B$26/12,Inputs!$B$27*12,-B68)))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A68&lt;Inputs!$B$28,Inputs!$B$27/12*B68,PMT(Inputs!$B$27/12,Inputs!$B$28*12,-B68)))</f>
         <v/>
       </c>
       <c r="D68" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,B68*Inputs!$B$26/12)</f>
+        <f>IF(Inputs!$B$49="Yes",0,B68*Inputs!$B$27/12)</f>
         <v/>
       </c>
       <c r="E68" s="17">
@@ -16914,19 +16914,19 @@
         <v/>
       </c>
       <c r="G68" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A68=Inputs!$B$30,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A68=Inputs!$B$31,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
         <v/>
       </c>
       <c r="H68" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A68=Inputs!$B$30,G68*Inputs!$B$31,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A68=Inputs!$B$31,G68*Inputs!$B$31,0))</f>
         <v/>
       </c>
       <c r="I68" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A68=Inputs!$B$30,MAX(0,H68-F68),0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A68=Inputs!$B$31,MAX(0,H68-F68),0))</f>
         <v/>
       </c>
       <c r="J68" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A68=Inputs!$B$30,H68,F68))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A68=Inputs!$B$31,H68,F68))</f>
         <v/>
       </c>
       <c r="K68" s="1" t="n"/>
@@ -16941,11 +16941,11 @@
         <v/>
       </c>
       <c r="C69" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A69&lt;Inputs!$B$28,Inputs!$B$26/12*B69,PMT(Inputs!$B$26/12,Inputs!$B$27*12,-B69)))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A69&lt;Inputs!$B$28,Inputs!$B$27/12*B69,PMT(Inputs!$B$27/12,Inputs!$B$28*12,-B69)))</f>
         <v/>
       </c>
       <c r="D69" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,B69*Inputs!$B$26/12)</f>
+        <f>IF(Inputs!$B$49="Yes",0,B69*Inputs!$B$27/12)</f>
         <v/>
       </c>
       <c r="E69" s="17">
@@ -16957,19 +16957,19 @@
         <v/>
       </c>
       <c r="G69" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A69=Inputs!$B$30,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A69=Inputs!$B$31,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
         <v/>
       </c>
       <c r="H69" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A69=Inputs!$B$30,G69*Inputs!$B$31,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A69=Inputs!$B$31,G69*Inputs!$B$31,0))</f>
         <v/>
       </c>
       <c r="I69" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A69=Inputs!$B$30,MAX(0,H69-F69),0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A69=Inputs!$B$31,MAX(0,H69-F69),0))</f>
         <v/>
       </c>
       <c r="J69" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A69=Inputs!$B$30,H69,F69))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A69=Inputs!$B$31,H69,F69))</f>
         <v/>
       </c>
       <c r="K69" s="1" t="n"/>
@@ -16984,11 +16984,11 @@
         <v/>
       </c>
       <c r="C70" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A70&lt;Inputs!$B$28,Inputs!$B$26/12*B70,PMT(Inputs!$B$26/12,Inputs!$B$27*12,-B70)))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A70&lt;Inputs!$B$28,Inputs!$B$27/12*B70,PMT(Inputs!$B$27/12,Inputs!$B$28*12,-B70)))</f>
         <v/>
       </c>
       <c r="D70" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,B70*Inputs!$B$26/12)</f>
+        <f>IF(Inputs!$B$49="Yes",0,B70*Inputs!$B$27/12)</f>
         <v/>
       </c>
       <c r="E70" s="17">
@@ -17000,19 +17000,19 @@
         <v/>
       </c>
       <c r="G70" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A70=Inputs!$B$30,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A70=Inputs!$B$31,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
         <v/>
       </c>
       <c r="H70" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A70=Inputs!$B$30,G70*Inputs!$B$31,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A70=Inputs!$B$31,G70*Inputs!$B$31,0))</f>
         <v/>
       </c>
       <c r="I70" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A70=Inputs!$B$30,MAX(0,H70-F70),0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A70=Inputs!$B$31,MAX(0,H70-F70),0))</f>
         <v/>
       </c>
       <c r="J70" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A70=Inputs!$B$30,H70,F70))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A70=Inputs!$B$31,H70,F70))</f>
         <v/>
       </c>
       <c r="K70" s="1" t="n"/>
@@ -17027,11 +17027,11 @@
         <v/>
       </c>
       <c r="C71" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A71&lt;Inputs!$B$28,Inputs!$B$26/12*B71,PMT(Inputs!$B$26/12,Inputs!$B$27*12,-B71)))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A71&lt;Inputs!$B$28,Inputs!$B$27/12*B71,PMT(Inputs!$B$27/12,Inputs!$B$28*12,-B71)))</f>
         <v/>
       </c>
       <c r="D71" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,B71*Inputs!$B$26/12)</f>
+        <f>IF(Inputs!$B$49="Yes",0,B71*Inputs!$B$27/12)</f>
         <v/>
       </c>
       <c r="E71" s="17">
@@ -17043,19 +17043,19 @@
         <v/>
       </c>
       <c r="G71" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A71=Inputs!$B$30,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A71=Inputs!$B$31,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
         <v/>
       </c>
       <c r="H71" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A71=Inputs!$B$30,G71*Inputs!$B$31,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A71=Inputs!$B$31,G71*Inputs!$B$31,0))</f>
         <v/>
       </c>
       <c r="I71" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A71=Inputs!$B$30,MAX(0,H71-F71),0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A71=Inputs!$B$31,MAX(0,H71-F71),0))</f>
         <v/>
       </c>
       <c r="J71" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A71=Inputs!$B$30,H71,F71))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A71=Inputs!$B$31,H71,F71))</f>
         <v/>
       </c>
       <c r="K71" s="1" t="n"/>
@@ -17070,11 +17070,11 @@
         <v/>
       </c>
       <c r="C72" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A72&lt;Inputs!$B$28,Inputs!$B$26/12*B72,PMT(Inputs!$B$26/12,Inputs!$B$27*12,-B72)))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A72&lt;Inputs!$B$28,Inputs!$B$27/12*B72,PMT(Inputs!$B$27/12,Inputs!$B$28*12,-B72)))</f>
         <v/>
       </c>
       <c r="D72" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,B72*Inputs!$B$26/12)</f>
+        <f>IF(Inputs!$B$49="Yes",0,B72*Inputs!$B$27/12)</f>
         <v/>
       </c>
       <c r="E72" s="17">
@@ -17086,19 +17086,19 @@
         <v/>
       </c>
       <c r="G72" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A72=Inputs!$B$30,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A72=Inputs!$B$31,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
         <v/>
       </c>
       <c r="H72" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A72=Inputs!$B$30,G72*Inputs!$B$31,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A72=Inputs!$B$31,G72*Inputs!$B$31,0))</f>
         <v/>
       </c>
       <c r="I72" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A72=Inputs!$B$30,MAX(0,H72-F72),0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A72=Inputs!$B$31,MAX(0,H72-F72),0))</f>
         <v/>
       </c>
       <c r="J72" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A72=Inputs!$B$30,H72,F72))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A72=Inputs!$B$31,H72,F72))</f>
         <v/>
       </c>
       <c r="K72" s="1" t="n"/>
@@ -17113,11 +17113,11 @@
         <v/>
       </c>
       <c r="C73" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A73&lt;Inputs!$B$28,Inputs!$B$26/12*B73,PMT(Inputs!$B$26/12,Inputs!$B$27*12,-B73)))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A73&lt;Inputs!$B$28,Inputs!$B$27/12*B73,PMT(Inputs!$B$27/12,Inputs!$B$28*12,-B73)))</f>
         <v/>
       </c>
       <c r="D73" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,B73*Inputs!$B$26/12)</f>
+        <f>IF(Inputs!$B$49="Yes",0,B73*Inputs!$B$27/12)</f>
         <v/>
       </c>
       <c r="E73" s="17">
@@ -17129,19 +17129,19 @@
         <v/>
       </c>
       <c r="G73" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A73=Inputs!$B$30,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A73=Inputs!$B$31,('Operating Expenses'!D17*4)/Inputs!$B$35,0))</f>
         <v/>
       </c>
       <c r="H73" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A73=Inputs!$B$30,G73*Inputs!$B$31,0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A73=Inputs!$B$31,G73*Inputs!$B$31,0))</f>
         <v/>
       </c>
       <c r="I73" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A73=Inputs!$B$30,MAX(0,H73-F73),0))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A73=Inputs!$B$31,MAX(0,H73-F73),0))</f>
         <v/>
       </c>
       <c r="J73" s="4">
-        <f>IF(Inputs!$B$49="Yes",0,IF(A73=Inputs!$B$30,H73,F73))</f>
+        <f>IF(Inputs!$B$49="Yes",0,IF(A73=Inputs!$B$31,H73,F73))</f>
         <v/>
       </c>
       <c r="K73" s="1" t="n"/>

</xml_diff>